<commit_message>
Control Hub Housing, H&S PCB
</commit_message>
<xml_diff>
--- a/Bill of Materials.xlsx
+++ b/Bill of Materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rphj0\Desktop\UW\Pozzo Lab\Science Jubilee Modular Equipment System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8722FFDE-E035-4F03-9EA5-FF955C301BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E605A9-39F3-4FBF-883E-3A12277E0354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="H&amp;S Module" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
   <si>
     <t>Motor</t>
   </si>
@@ -152,6 +152,45 @@
   </si>
   <si>
     <t>Fan</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/sunon-fans/MF40100V1-1000U-A99/6198732</t>
+  </si>
+  <si>
+    <t>2x2 Conn</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/molex/0039012041/61227</t>
+  </si>
+  <si>
+    <t>USB</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.us/item/3256807073804695.html?gatewayAdapt=glo2usa</t>
+  </si>
+  <si>
+    <t>3-state SW</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/adam-tech/SW-T2-2E-A-A2-M1/15284450</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/e-switch/PS1024ARED/44577</t>
+  </si>
+  <si>
+    <t>Ill on/off SW</t>
+  </si>
+  <si>
+    <t>https://switches-sensors.zf.com/wp-content/uploads/2024/08/Rocker_SRB_Datasheet_2024-08-02.pdf</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>3mm diam</t>
   </si>
 </sst>
 </file>
@@ -637,7 +676,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29CF2ED5-99EB-4A54-8082-842D732B373B}">
-  <dimension ref="A3:C8"/>
+  <dimension ref="A3:C14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.46484375" customWidth="1"/>
@@ -681,6 +720,57 @@
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -745,19 +835,19 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>0.15</v>
+        <v>0.23499999999999999</v>
       </c>
       <c r="D4">
         <f>B4*C4</f>
-        <v>1.7999999999999998</v>
+        <v>2.82</v>
       </c>
       <c r="E4">
         <f>D4*B1</f>
-        <v>9</v>
+        <v>14.1</v>
       </c>
       <c r="F4">
         <f>E4*B2</f>
-        <v>54</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -768,20 +858,20 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <f>B1/6.48</f>
-        <v>0.77160493827160492</v>
+        <f>B1/1.67</f>
+        <v>2.9940119760479043</v>
       </c>
       <c r="D5">
         <f>B5*C5</f>
-        <v>3.0864197530864197</v>
+        <v>11.976047904191617</v>
       </c>
       <c r="E5">
-        <f>B1*D5</f>
-        <v>15.432098765432098</v>
+        <f>15*4</f>
+        <v>60</v>
       </c>
       <c r="F5">
         <f>E5*B2</f>
-        <v>92.592592592592581</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -790,7 +880,7 @@
       </c>
       <c r="F7">
         <f>F4+F5</f>
-        <v>146.59259259259258</v>
+        <v>444.6</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -799,7 +889,7 @@
       </c>
       <c r="F8">
         <f>F7/5</f>
-        <v>29.318518518518516</v>
+        <v>88.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>